<commit_message>
Autónomos: importar los modelos 111 y 115 presentados (PDF), sus plantillas y los ejemplos con retenciones
El lector de modelos reconoce el 111 y el 115 por su título y sus casillas (01-30 y 01-05);
al importarlos, sus empleados, profesionales o alquiler rellenan las retenciones de ese
trimestre, marcadas como importadas, y las facturas de ese trimestre dejan de sumarse.
Plantillas PDF rellenables del 111 y el 115 para descargar. El libro de facturas recibidas de
ejemplo trae la retención del alquiler del local (19 %), la gestoría (15 %) y una diseñadora
(7 %), con el NIF; hay un ejemplo de empleados y el 111 y el 115 del 2T rellenados.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/ejemplos-importacion/ejemplo-facturas-recibidas-2026.xlsx
+++ b/docs/ejemplos-importacion/ejemplo-facturas-recibidas-2026.xlsx
@@ -8,7 +8,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="16" uniqueCount="16">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="23" uniqueCount="23">
   <si>
     <t xml:space="preserve">Libro registro de facturas recibidas · ejemplo con datos inventados</t>
   </si>
@@ -31,10 +31,31 @@
     <t xml:space="preserve">Cuota IVA Soportado</t>
   </si>
   <si>
-    <t xml:space="preserve">Alquiler oficina coworking</t>
+    <t xml:space="preserve">NIF Expedidor</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Tipo Retención IRPF</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Importe Retenido IRPF</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Inmuebles Ribera SL alquiler del local</t>
+  </si>
+  <si>
+    <t xml:space="preserve">B00000001</t>
   </si>
   <si>
     <t xml:space="preserve">Gestoría Pérez asesoría fiscal</t>
+  </si>
+  <si>
+    <t xml:space="preserve">00000001R</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Marta Ejemplo diseño gráfico</t>
+  </si>
+  <si>
+    <t xml:space="preserve">00000002W</t>
   </si>
   <si>
     <t xml:space="preserve">Adobe licencia software</t>
@@ -129,16 +150,25 @@
       <c r="F4" t="s">
         <v>6</v>
       </c>
+      <c r="G4" t="s">
+        <v>7</v>
+      </c>
+      <c r="H4" t="s">
+        <v>8</v>
+      </c>
+      <c r="I4" t="s">
+        <v>9</v>
+      </c>
     </row>
     <row r="5">
       <c r="A5" s="1">
         <v>46027</v>
       </c>
       <c r="B5" t="s">
-        <v>7</v>
+        <v>10</v>
       </c>
       <c r="C5">
-        <v>484</v>
+        <v>408</v>
       </c>
       <c r="D5">
         <v>400</v>
@@ -148,6 +178,15 @@
       </c>
       <c r="F5">
         <v>84</v>
+      </c>
+      <c r="G5" t="s">
+        <v>11</v>
+      </c>
+      <c r="H5">
+        <v>19</v>
+      </c>
+      <c r="I5">
+        <v>76</v>
       </c>
     </row>
     <row r="6">
@@ -155,10 +194,10 @@
         <v>46063</v>
       </c>
       <c r="B6" t="s">
-        <v>8</v>
+        <v>12</v>
       </c>
       <c r="C6">
-        <v>181.5</v>
+        <v>159</v>
       </c>
       <c r="D6">
         <v>150</v>
@@ -169,273 +208,345 @@
       <c r="F6">
         <v>31.5</v>
       </c>
+      <c r="G6" t="s">
+        <v>13</v>
+      </c>
+      <c r="H6">
+        <v>15</v>
+      </c>
+      <c r="I6">
+        <v>22.5</v>
+      </c>
     </row>
     <row r="7">
       <c r="A7" s="1">
-        <v>46117</v>
+        <v>46073</v>
       </c>
       <c r="B7" t="s">
+        <v>14</v>
+      </c>
+      <c r="C7">
+        <v>57</v>
+      </c>
+      <c r="D7">
+        <v>50</v>
+      </c>
+      <c r="E7">
+        <v>21</v>
+      </c>
+      <c r="F7">
+        <v>10.5</v>
+      </c>
+      <c r="G7" t="s">
+        <v>15</v>
+      </c>
+      <c r="H7">
         <v>7</v>
       </c>
-      <c r="C7">
-        <v>484</v>
-      </c>
-      <c r="D7">
-        <v>400</v>
-      </c>
-      <c r="E7">
-        <v>21</v>
-      </c>
-      <c r="F7">
-        <v>84</v>
+      <c r="I7">
+        <v>3.5</v>
       </c>
     </row>
     <row r="8">
       <c r="A8" s="1">
-        <v>46152</v>
+        <v>46117</v>
       </c>
       <c r="B8" t="s">
-        <v>8</v>
+        <v>10</v>
       </c>
       <c r="C8">
-        <v>181.5</v>
+        <v>408</v>
       </c>
       <c r="D8">
-        <v>150</v>
+        <v>400</v>
       </c>
       <c r="E8">
         <v>21</v>
       </c>
       <c r="F8">
-        <v>31.5</v>
+        <v>84</v>
+      </c>
+      <c r="G8" t="s">
+        <v>11</v>
+      </c>
+      <c r="H8">
+        <v>19</v>
+      </c>
+      <c r="I8">
+        <v>76</v>
       </c>
     </row>
     <row r="9">
       <c r="A9" s="1">
-        <v>46208</v>
+        <v>46152</v>
       </c>
       <c r="B9" t="s">
-        <v>7</v>
+        <v>12</v>
       </c>
       <c r="C9">
-        <v>484</v>
+        <v>159</v>
       </c>
       <c r="D9">
-        <v>400</v>
+        <v>150</v>
       </c>
       <c r="E9">
         <v>21</v>
       </c>
       <c r="F9">
-        <v>84</v>
+        <v>31.5</v>
+      </c>
+      <c r="G9" t="s">
+        <v>13</v>
+      </c>
+      <c r="H9">
+        <v>15</v>
+      </c>
+      <c r="I9">
+        <v>22.5</v>
       </c>
     </row>
     <row r="10">
       <c r="A10" s="1">
-        <v>46244</v>
+        <v>46162</v>
       </c>
       <c r="B10" t="s">
-        <v>8</v>
+        <v>14</v>
       </c>
       <c r="C10">
-        <v>181.5</v>
+        <v>57</v>
       </c>
       <c r="D10">
-        <v>150</v>
+        <v>50</v>
       </c>
       <c r="E10">
         <v>21</v>
       </c>
       <c r="F10">
-        <v>31.5</v>
+        <v>10.5</v>
+      </c>
+      <c r="G10" t="s">
+        <v>15</v>
+      </c>
+      <c r="H10">
+        <v>7</v>
+      </c>
+      <c r="I10">
+        <v>3.5</v>
       </c>
     </row>
     <row r="11">
       <c r="A11" s="1">
-        <v>46042</v>
+        <v>46208</v>
       </c>
       <c r="B11" t="s">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="C11">
-        <v>72.6</v>
+        <v>408</v>
       </c>
       <c r="D11">
-        <v>60</v>
+        <v>400</v>
       </c>
       <c r="E11">
         <v>21</v>
       </c>
       <c r="F11">
-        <v>12.6</v>
+        <v>84</v>
+      </c>
+      <c r="G11" t="s">
+        <v>11</v>
+      </c>
+      <c r="H11">
+        <v>19</v>
+      </c>
+      <c r="I11">
+        <v>76</v>
       </c>
     </row>
     <row r="12">
       <c r="A12" s="1">
-        <v>46067</v>
+        <v>46244</v>
       </c>
       <c r="B12" t="s">
-        <v>10</v>
+        <v>12</v>
       </c>
       <c r="C12">
-        <v>96.8</v>
+        <v>159</v>
       </c>
       <c r="D12">
-        <v>80</v>
+        <v>150</v>
       </c>
       <c r="E12">
         <v>21</v>
       </c>
       <c r="F12">
-        <v>16.8</v>
+        <v>31.5</v>
+      </c>
+      <c r="G12" t="s">
+        <v>13</v>
+      </c>
+      <c r="H12">
+        <v>15</v>
+      </c>
+      <c r="I12">
+        <v>22.5</v>
       </c>
     </row>
     <row r="13">
       <c r="A13" s="1">
-        <v>46134</v>
+        <v>46254</v>
       </c>
       <c r="B13" t="s">
-        <v>11</v>
+        <v>14</v>
       </c>
       <c r="C13">
-        <v>145.2</v>
+        <v>57</v>
       </c>
       <c r="D13">
-        <v>120</v>
+        <v>50</v>
       </c>
       <c r="E13">
         <v>21</v>
       </c>
       <c r="F13">
-        <v>25.2</v>
+        <v>10.5</v>
+      </c>
+      <c r="G13" t="s">
+        <v>15</v>
+      </c>
+      <c r="H13">
+        <v>7</v>
+      </c>
+      <c r="I13">
+        <v>3.5</v>
       </c>
     </row>
     <row r="14">
       <c r="A14" s="1">
-        <v>46172</v>
+        <v>46042</v>
       </c>
       <c r="B14" t="s">
-        <v>12</v>
+        <v>16</v>
       </c>
       <c r="C14">
-        <v>60.5</v>
+        <v>72.6</v>
       </c>
       <c r="D14">
-        <v>55</v>
+        <v>60</v>
       </c>
       <c r="E14">
-        <v>10</v>
+        <v>21</v>
       </c>
       <c r="F14">
-        <v>5.5</v>
+        <v>12.6</v>
       </c>
     </row>
     <row r="15">
       <c r="A15" s="1">
-        <v>46252</v>
+        <v>46067</v>
       </c>
       <c r="B15" t="s">
-        <v>13</v>
+        <v>17</v>
       </c>
       <c r="C15">
-        <v>363</v>
+        <v>96.8</v>
       </c>
       <c r="D15">
-        <v>300</v>
+        <v>80</v>
       </c>
       <c r="E15">
         <v>21</v>
       </c>
       <c r="F15">
-        <v>63</v>
+        <v>16.8</v>
       </c>
     </row>
     <row r="16">
       <c r="A16" s="1">
-        <v>46268</v>
+        <v>46134</v>
       </c>
       <c r="B16" t="s">
-        <v>14</v>
+        <v>18</v>
       </c>
       <c r="C16">
-        <v>108.9</v>
+        <v>145.2</v>
       </c>
       <c r="D16">
-        <v>90</v>
+        <v>120</v>
       </c>
       <c r="E16">
         <v>21</v>
       </c>
       <c r="F16">
-        <v>18.9</v>
+        <v>25.2</v>
       </c>
     </row>
     <row r="17">
       <c r="A17" s="1">
-        <v>46050</v>
+        <v>46172</v>
       </c>
       <c r="B17" t="s">
-        <v>15</v>
+        <v>19</v>
       </c>
       <c r="C17">
-        <v>294</v>
+        <v>60.5</v>
       </c>
       <c r="D17">
-        <v>294</v>
+        <v>55</v>
       </c>
       <c r="E17">
-        <v>0</v>
+        <v>10</v>
       </c>
       <c r="F17">
-        <v>0</v>
+        <v>5.5</v>
       </c>
     </row>
     <row r="18">
       <c r="A18" s="1">
-        <v>46081</v>
+        <v>46252</v>
       </c>
       <c r="B18" t="s">
-        <v>15</v>
+        <v>20</v>
       </c>
       <c r="C18">
-        <v>294</v>
+        <v>363</v>
       </c>
       <c r="D18">
-        <v>294</v>
+        <v>300</v>
       </c>
       <c r="E18">
-        <v>0</v>
+        <v>21</v>
       </c>
       <c r="F18">
-        <v>0</v>
+        <v>63</v>
       </c>
     </row>
     <row r="19">
       <c r="A19" s="1">
-        <v>46109</v>
+        <v>46268</v>
       </c>
       <c r="B19" t="s">
-        <v>15</v>
+        <v>21</v>
       </c>
       <c r="C19">
-        <v>294</v>
+        <v>108.9</v>
       </c>
       <c r="D19">
-        <v>294</v>
+        <v>90</v>
       </c>
       <c r="E19">
-        <v>0</v>
+        <v>21</v>
       </c>
       <c r="F19">
-        <v>0</v>
+        <v>18.9</v>
       </c>
     </row>
     <row r="20">
       <c r="A20" s="1">
-        <v>46140</v>
+        <v>46050</v>
       </c>
       <c r="B20" t="s">
-        <v>15</v>
+        <v>22</v>
       </c>
       <c r="C20">
         <v>294</v>
@@ -452,10 +563,10 @@
     </row>
     <row r="21">
       <c r="A21" s="1">
-        <v>46170</v>
+        <v>46081</v>
       </c>
       <c r="B21" t="s">
-        <v>15</v>
+        <v>22</v>
       </c>
       <c r="C21">
         <v>294</v>
@@ -472,10 +583,10 @@
     </row>
     <row r="22">
       <c r="A22" s="1">
-        <v>46201</v>
+        <v>46109</v>
       </c>
       <c r="B22" t="s">
-        <v>15</v>
+        <v>22</v>
       </c>
       <c r="C22">
         <v>294</v>
@@ -492,10 +603,10 @@
     </row>
     <row r="23">
       <c r="A23" s="1">
-        <v>46231</v>
+        <v>46140</v>
       </c>
       <c r="B23" t="s">
-        <v>15</v>
+        <v>22</v>
       </c>
       <c r="C23">
         <v>294</v>
@@ -512,10 +623,10 @@
     </row>
     <row r="24">
       <c r="A24" s="1">
-        <v>46262</v>
+        <v>46170</v>
       </c>
       <c r="B24" t="s">
-        <v>15</v>
+        <v>22</v>
       </c>
       <c r="C24">
         <v>294</v>
@@ -532,21 +643,81 @@
     </row>
     <row r="25">
       <c r="A25" s="1">
+        <v>46201</v>
+      </c>
+      <c r="B25" t="s">
+        <v>22</v>
+      </c>
+      <c r="C25">
+        <v>294</v>
+      </c>
+      <c r="D25">
+        <v>294</v>
+      </c>
+      <c r="E25">
+        <v>0</v>
+      </c>
+      <c r="F25">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" s="1">
+        <v>46231</v>
+      </c>
+      <c r="B26" t="s">
+        <v>22</v>
+      </c>
+      <c r="C26">
+        <v>294</v>
+      </c>
+      <c r="D26">
+        <v>294</v>
+      </c>
+      <c r="E26">
+        <v>0</v>
+      </c>
+      <c r="F26">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" s="1">
+        <v>46262</v>
+      </c>
+      <c r="B27" t="s">
+        <v>22</v>
+      </c>
+      <c r="C27">
+        <v>294</v>
+      </c>
+      <c r="D27">
+        <v>294</v>
+      </c>
+      <c r="E27">
+        <v>0</v>
+      </c>
+      <c r="F27">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" s="1">
         <v>46293</v>
       </c>
-      <c r="B25" t="s">
-        <v>15</v>
-      </c>
-      <c r="C25">
-        <v>294</v>
-      </c>
-      <c r="D25">
-        <v>294</v>
-      </c>
-      <c r="E25">
-        <v>0</v>
-      </c>
-      <c r="F25">
+      <c r="B28" t="s">
+        <v>22</v>
+      </c>
+      <c r="C28">
+        <v>294</v>
+      </c>
+      <c r="D28">
+        <v>294</v>
+      </c>
+      <c r="E28">
+        <v>0</v>
+      </c>
+      <c r="F28">
         <v>0</v>
       </c>
     </row>

</xml_diff>